<commit_message>
versione finale updated self assessment
</commit_message>
<xml_diff>
--- a/Fresh Carrots/Self Assessment Form - IUM-TWEB.xlsx
+++ b/Fresh Carrots/Self Assessment Form - IUM-TWEB.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabrielebuoso/Desktop/Consegna TWEB/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabrielebuoso/Desktop/TWEB_2425/Fresh Carrots/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6FF84FE-7EDA-C343-A9D3-C680D5CFC5C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53862FAA-943F-F84E-9FB8-7A2F685512CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="660" windowWidth="38100" windowHeight="20800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -204,9 +204,6 @@
     <t xml:space="preserve">La nostra idea di implementazione non prevede la possibilità di aggiungere dati sul DB Postgres. Il retrieve funziona correttamente </t>
   </si>
   <si>
-    <t>Abbiamo utilizzato lo standard OpenAPI con swagger per i tre server (server express on /api-docs, springboot on /swagger-ui/index.html).</t>
-  </si>
-  <si>
     <t>Per la visualizzazzione di recensioni nella pagina Reviews, film nella pagina Discover e per il caricamento di messaggi nella pagina DiscussionRoom abbiamo implementato una query paginata integrata con infinte scroll. I messaggi inoltre, vengono salvati sul database dinamico MongoDB.</t>
   </si>
   <si>
@@ -223,6 +220,9 @@
   </si>
   <si>
     <t>Lavorando in contemporanea con il compagno il lavoro è stato diviso equamente tra le parti, però più specificamente si è occupato di: sviluppo React in particolare sulla parte di efficienza e comunicazione con il il main server. Main Server Express:gestione degli errori e la definizione della comunicazione socket based. Springboot più sulle Specifications e lo sviluppo dei metodi nelle repository. Dynamic Express Server: definizione degli schemas, efficienza nelle query ed error handling. Più in generale l'ideazione e lo sviluppo degli endpoint in tutti i server, e proprosition di idee innovative. Ci teniamo a precisare che le parti hanno collaborato in egual modo, sempre in contatto su Meet o Discord, assegnamo dunque esattamente la metà del carico del lavoro a ciascuno.</t>
+  </si>
+  <si>
+    <t>Abbiamo utilizzato lo standard OpenAPI con swagger per i tre server (server express on /api-docs, springboot on /swagger-ui/index.html). Inoltre il codice è commentato in notazione javadoc per ogni funzione del Frontend React, così come Dynamic Express Server, mentre per Java SpringBoot nelle funzioni di supporto non tracciate dallo swagger.</t>
   </si>
 </sst>
 </file>
@@ -540,6 +540,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -549,10 +553,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="9" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -780,12 +780,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="94.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="46"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
@@ -810,12 +810,12 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="64.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -1253,7 +1253,7 @@
         <v>24</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1341,7 +1341,7 @@
         <v>24</v>
       </c>
       <c r="C55" s="10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1392,7 +1392,7 @@
         <v>24</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1421,7 +1421,7 @@
       <c r="D65" s="14">
         <v>3</v>
       </c>
-      <c r="E65" s="48" t="s">
+      <c r="E65" s="43" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1443,13 +1443,13 @@
         <v>4</v>
       </c>
     </row>
-    <row r="68" spans="1:5" ht="72" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" ht="162" x14ac:dyDescent="0.25">
       <c r="A68" s="23"/>
       <c r="B68" s="24" t="s">
         <v>24</v>
       </c>
       <c r="C68" s="10" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1468,7 +1468,7 @@
         <v>46</v>
       </c>
       <c r="C71" s="41" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1500,10 +1500,10 @@
         <v>48</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D75" s="10"/>
     </row>
@@ -1511,10 +1511,10 @@
       <c r="A76" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="B76" s="47">
+      <c r="B76" s="42">
         <v>0.5</v>
       </c>
-      <c r="C76" s="47">
+      <c r="C76" s="42">
         <v>0.5</v>
       </c>
       <c r="D76" s="25"/>

</xml_diff>